<commit_message>
docs: Cap nhat day du thong tin 3 thanh vien Nhom 2 lop KTPM K23B vao README, Docs va Excel
</commit_message>
<xml_diff>
--- a/BANG_KIEM_THU_VA_FIX_LOI_SMARTLIB.xlsx
+++ b/BANG_KIEM_THU_VA_FIX_LOI_SMARTLIB.xlsx
@@ -668,7 +668,7 @@
     <row r="2" ht="19.95" customHeight="1" s="17">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Tự động hóa 100% trong test_evaluation.py (Thời gian chạy: 1.47 giây | Tỷ lệ thành công: 40/40 PASS - 100%)</t>
+          <t>Lớp: KTPM K23B | Nhóm SV: Vũ Hồng Dũng (Trưởng nhóm - DTC245180068), Nguyễn Trung Học (DTC245180174), Lê Quang Hưng (DTC245180036)</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
     <row r="2" ht="19.95" customHeight="1" s="17">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Dành cho đội ngũ Backend, Frontend, DevOps đối chiếu nguyên nhân và cách xử lý trong mã nguồn</t>
+          <t>Lớp: KTPM K23B | Nhóm SV: Vũ Hồng Dũng (Trưởng nhóm - DTC245180068), Nguyễn Trung Học (DTC245180174), Lê Quang Hưng (DTC245180036)</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,11 @@
       </c>
     </row>
     <row r="2" ht="19.95" customHeight="1" s="17">
-      <c r="A2" s="16" t="n"/>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Lớp: KTPM K23B | Nhóm SV: Vũ Hồng Dũng (Trưởng nhóm - DTC245180068), Nguyễn Trung Học (DTC245180174), Lê Quang Hưng (DTC245180036)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="10.05" customHeight="1" s="17"/>
     <row r="4" ht="30" customHeight="1" s="17">

</xml_diff>